<commit_message>
UPDATED : El gato version, rsync after cgMLST extract, Kraken with Qiime2
</commit_message>
<xml_diff>
--- a/Pipeline_assembly_mlst/assets/MLST_Assembly_metadata.xlsx
+++ b/Pipeline_assembly_mlst/assets/MLST_Assembly_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\04_CNR_Legionella\Input_analysis_nextflow\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D465634-E223-4944-BF14-835B4F0BAEED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{048378AF-48BF-49C8-972E-ACB9D70D31EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B3C5F1E1-92BF-4413-A239-65E07C6C183A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{B3C5F1E1-92BF-4413-A239-65E07C6C183A}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -124,63 +124,6 @@
   </si>
   <si>
     <r>
-      <t>Origin</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> : origine de l’échantillon. Valeurs autorisées : </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Clinical</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> ou </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Environment</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (exactement ces termes).</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">La feuille </t>
     </r>
     <r>
@@ -285,63 +228,6 @@
   </si>
   <si>
     <r>
-      <t>Origin</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: sample source. Allowed values: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Clinical</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> or </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Environment</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (exact strings).</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">The </t>
     </r>
     <r>
@@ -389,38 +275,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Le nom du fichier doit respecter la règle suivante : </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Metadata_YYYYMMDD.tsv</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The file name must follow this pattern: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Metadata_YYYYMMDD.tsv</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <rPr>
         <b/>
         <sz val="12"/>
@@ -507,6 +361,42 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> corresponds to the sequencing date (as written in NGS-WEB).</t>
+    </r>
+  </si>
+  <si>
+    <t>/!\ Le fichier doit être enregistré au chemin suivant : TMP_IAI\04_CNR_Legionella\Input_analysis_nextflow</t>
+  </si>
+  <si>
+    <t>/!\ The file must be saved to the following path: TMP_IAI\04_CNR_Legionella\Input_analysis_nextflow</t>
+  </si>
+  <si>
+    <r>
+      <t>Linked_to</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : lien vers un autre identifiant. Longueur 6 à 100 caractères, seuls lettres, chiffres et « - » autorisés.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Linked_to</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: reference to another ID. Length 6–100 characters, only letters, numbers, and “-” allowed.</t>
     </r>
   </si>
   <si>
@@ -564,7 +454,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Metadata_YYYYMMDD.tsv</t>
+      <t>Metadata_YYYYMMDD.txt</t>
     </r>
     <r>
       <rPr>
@@ -579,6 +469,38 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">Le nom du fichier doit respecter la règle suivante : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Metadata_YYYYMMDD.txt</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The file name must follow this pattern: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Metadata_YYYYMMDD.txt</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">In Excel, go to </t>
     </r>
     <r>
@@ -632,7 +554,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Metadata_YYYYMMDD.tsv</t>
+      <t>Metadata_YYYYMMDD.txt</t>
     </r>
     <r>
       <rPr>
@@ -646,40 +568,10 @@
     </r>
   </si>
   <si>
-    <t>/!\ Le fichier doit être enregistré au chemin suivant : TMP_IAI\04_CNR_Legionella\Input_analysis_nextflow</t>
-  </si>
-  <si>
-    <t>/!\ The file must be saved to the following path: TMP_IAI\04_CNR_Legionella\Input_analysis_nextflow</t>
-  </si>
-  <si>
-    <r>
-      <t>Linked_to</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> : lien vers un autre identifiant. Longueur 6 à 100 caractères, seuls lettres, chiffres et « - » autorisés.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Linked_to</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: reference to another ID. Length 6–100 characters, only letters, numbers, and “-” allowed.</t>
-    </r>
+    <t>Origin : origine de l’échantillon. Valeurs autorisées : Clinic ou Environment (exactement ces termes).</t>
+  </si>
+  <si>
+    <t>Origin: sample source. Allowed values: Clinic or Environment (exact strings).</t>
   </si>
 </sst>
 </file>
@@ -1313,10 +1205,10 @@
       <c r="D20" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" deleteRows="0"/>
+  <sheetProtection deleteRows="0"/>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Wrong value" error="Veuillez choisir une valeur entre &quot;Clinical&quot; ou &quot;Environment&quot; seulement. _x000a_---_x000a_Please select either ‘Clinical’ or ‘Environment’ only. " sqref="C1:C1048576" xr:uid="{7781F29C-D146-4AD2-8551-C45AC2B371AA}">
-      <formula1>"Clinical,Environment"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Wrong value" error="Veuillez choisir une valeur entre &quot;Clinic&quot; ou &quot;Environment&quot; seulement. _x000a_---_x000a_Please select either ‘Clinic’ or ‘Environment’ only. " sqref="C1:C1048576" xr:uid="{7781F29C-D146-4AD2-8551-C45AC2B371AA}">
+      <formula1>"Clinic,Environment"</formula1>
     </dataValidation>
     <dataValidation type="whole" showInputMessage="1" showErrorMessage="1" errorTitle="Wrong data format" error="Veuillez entrer l'année d'isolement/de récupération de l'échantillon au format YYYY._x000a_---_x000a_Please enter the year the sample was isolated/collected in the format YYYY." sqref="B1:B1048576" xr:uid="{5B5CF9F9-1897-4486-B33C-4A43570CE5F3}">
       <formula1>1900</formula1>
@@ -1349,7 +1241,7 @@
     </row>
     <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C5" s="17" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -1359,12 +1251,12 @@
     </row>
     <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C7" s="13" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C8" s="13" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="23.4" x14ac:dyDescent="0.3">
@@ -1377,7 +1269,7 @@
     </row>
     <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C13" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -1385,13 +1277,13 @@
     </row>
     <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C15" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C16" s="14"/>
       <c r="D16" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -1404,7 +1296,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D19" s="18" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -1424,22 +1316,22 @@
     </row>
     <row r="26" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C26" s="13" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C27" s="13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C28" s="13" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C29" s="13" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -1455,7 +1347,7 @@
     </row>
     <row r="34" spans="3:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C34" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="35" spans="3:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -1463,13 +1355,13 @@
     </row>
     <row r="36" spans="3:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C36" s="1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="37" spans="3:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C37" s="14"/>
       <c r="D37" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38" spans="3:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -1477,13 +1369,13 @@
     </row>
     <row r="39" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C39" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="40" spans="3:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="C40" s="1"/>
       <c r="D40" s="18" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>